<commit_message>
data: expand labs/professors coverage (LiDAR, 3D CV, environmental RS)
Adds ~34 new research groups spanning SLAM/robotics, deep-learning
photogrammetry, environmental & forest remote sensing, and more
Asia-Pacific/NA institutions. Labs now list responsible professors,
shown on the site's lab cards and included in search. tracker.xlsx
is the source of truth (Labs sheet gets a new Professors column);
data/*.json regenerated via crawler/excel_to_json.py.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/tracker.xlsx
+++ b/data/tracker.xlsx
@@ -2548,7 +2548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2622,653 +2622,1444 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Cyrill Stachniss</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>University of Bonn</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Photogrammetry &amp; Robotics Lab</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>SLAM; LiDAR Mapping; Photogrammetry</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Konrad Schindler</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>ETH Zurich</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Photogrammetry and Remote Sensing</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Photogrammetry; Computer Vision (2D/3D); GeoAI / Deep Learning</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Norbert Pfeifer</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>TU Wien</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Photogrammetry / Geodesy &amp; Geoinformation</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Austria</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>LiDAR Mapping; Forest LiDAR</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Juha Hyyppä</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Finnish Geospatial Research Institute (FGI)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Remote Sensing &amp; Photogrammetry</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Finland</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Forest LiDAR; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Ayman Habib</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Purdue University</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Digital Photogrammetry Research Group</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping; Adjustment &amp; Geodesy</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Xiaoxiang Zhu</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Technical University of Munich</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Data Science in Earth Observation</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>GeoAI / Deep Learning; Remote Sensing</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n"/>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Norbert Haala</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>University of Stuttgart</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Institute for Photogrammetry and Geoinformatics</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Seed entry — verify current affiliation and add links</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n"/>
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Christian Heipke</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Leibniz University Hannover</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Institute of Photogrammetry and GeoInformation</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Franz Rottensteiner</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Leibniz University Hannover</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Institute of Photogrammetry and GeoInformation</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n"/>
-      <c r="B11" s="3" t="n"/>
-      <c r="C11" s="3" t="n"/>
-      <c r="D11" s="3" t="n"/>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Juha Hyyppä</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>National Land Survey of Finland</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Finnish Geospatial Research Institute</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="n"/>
-      <c r="J12" s="2" t="n"/>
-      <c r="K12" s="2" t="n"/>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Naser El-Sheimy</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>University of Calgary</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Geomatics Engineering</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Adjustment &amp; Geodesy; LiDAR Mapping; SLAM</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n"/>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
-      <c r="D13" s="3" t="n"/>
-      <c r="E13" s="3" t="n"/>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Liangpei Zhang</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wuhan University</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>LIESMARS (Surveying, Mapping &amp; RS)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
-      <c r="H14" s="2" t="n"/>
-      <c r="I14" s="2" t="n"/>
-      <c r="J14" s="2" t="n"/>
-      <c r="K14" s="2" t="n"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Deren Li</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wuhan University</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>LIESMARS (Surveying, Mapping &amp; RS)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n"/>
-      <c r="B15" s="3" t="n"/>
-      <c r="C15" s="3" t="n"/>
-      <c r="D15" s="3" t="n"/>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bo Wu</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hong Kong Polytechnic University</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Land Surveying &amp; Geo-Informatics (LSGI)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hong Kong</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; Adjustment &amp; Geodesy</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-      <c r="K16" s="2" t="n"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Andreas Geiger</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>University of Tübingen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Autonomous Vision Group</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n"/>
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Daniel Cremers</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Computer Vision Group</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-      <c r="K18" s="2" t="n"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Marc Pollefeys</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Computer Vision and Geometry Group</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM; Photogrammetry</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n"/>
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Davide Scaramuzza</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>University of Zurich</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Robotics and Perception Group</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
-      <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-      <c r="K20" s="2" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Roland Siegwart</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Autonomous Systems Lab</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>SLAM; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Andrew Davison</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Imperial College London</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Dyson Robotics Lab</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
-      <c r="K22" s="2" t="n"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Stefan Leutenegger</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Smart Robotics Lab</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n"/>
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sebastian Scherer</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Air Lab</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>SLAM; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n"/>
-      <c r="K24" s="2" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Michael Kaess</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Robot Perception Lab</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Frank Dellaert</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Georgia Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Borglab</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Uwe Stilla</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Chair of Photogrammetry and Remote Sensing</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Photogrammetry; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bernhard Höfle</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Heidelberg University</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>3D Geospatial Data Processing Group (3DGeo)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
-      <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="n"/>
-      <c r="K28" s="2" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Stefan Hinz</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Karlsruhe Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Remote Sensing Image Analysis Group</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Boris Jutzi</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Karlsruhe Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Institute of Photogrammetry and Remote Sensing (IPF)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Computer Vision (2D/3D); Photogrammetry</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
-      <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="n"/>
-      <c r="K30" s="2" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Martin Weinmann</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Karlsruhe Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Institute of Photogrammetry and Remote Sensing (IPF)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Computer Vision (2D/3D); Photogrammetry</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Monika Sester</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Leibniz University Hannover</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Institute of Cartography and Geoinformatics</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>GeoAI / Deep Learning; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
-      <c r="I32" s="2" t="n"/>
-      <c r="J32" s="2" t="n"/>
-      <c r="K32" s="2" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jan Dirk Wegner</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>University of Zurich</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>EcoVision Lab</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning; Forest LiDAR</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Devis Tuia</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Environmental Computational Science and Earth Observation Lab (ECEO)</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="n"/>
-      <c r="J34" s="2" t="n"/>
-      <c r="K34" s="2" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Gustau Camps-Valls</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>University of Valencia</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Image Processing Laboratory (IPL)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Barbara Koch</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>University of Freiburg</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Chair of Remote Sensing and Landscape Information Systems</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
-      <c r="I36" s="2" t="n"/>
-      <c r="J36" s="2" t="n"/>
-      <c r="K36" s="2" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Erik Næsset</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Norwegian University of Life Sciences (NMBU)</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Faculty of Environmental Sciences and Natural Resource Management</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Terje Gobakken</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Norwegian University of Life Sciences (NMBU)</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Faculty of Environmental Sciences and Natural Resource Management</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Mikko Vastaranta</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>University of Helsinki</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Department of Forest Sciences</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Markus Reichstein</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Max Planck Institute for Biogeochemistry</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Department of Biogeochemical Integration</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Ross Meentemeyer</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>North Carolina State University</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Center for Geospatial Analytics</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Nico Sneeuw</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>University of Stuttgart</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Institute of Geodesy</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Adjustment &amp; Geodesy</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Huadong Guo</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Chinese Academy of Sciences</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Institute of Remote Sensing and Digital Earth (RADI)</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Ryosuke Shibasaki</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>University of Tokyo</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Department of Geoinformatics</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Linlin Ge</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>School of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Adjustment &amp; Geodesy; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Jinha Jung</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Purdue University</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Digital Photogrammetry Research Group</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Benjamin Wu</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>University of Florida</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Geospatial Data Analysis Lab</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and add links</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3282,7 +4073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3317,1013 +4108,2312 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Professors</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Typical Intake</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Photogrammetry &amp; Robotics Lab</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>University of Bonn</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>SLAM; LiDAR Mapping; Photogrammetry</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cyrill Stachniss</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://www.uni-bonn.de</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Photogrammetry and Remote Sensing (IGP)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>ETH Zurich</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Photogrammetry; GeoAI / Deep Learning; Computer Vision (2D/3D)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Konrad Schindler</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://ethz.ch</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Institute for Photogrammetry and Geoinformatics</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>University of Stuttgart</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Norbert Haala</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.uni-stuttgart.de</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Data Science in Earth Observation</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Technical University of Munich</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>GeoAI / Deep Learning; Remote Sensing</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Xiaoxiang Zhu</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.tum.de</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Institute of Photogrammetry and GeoInformation</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Leibniz University Hannover</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping; Computer Vision (2D/3D)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Christian Heipke; Franz Rottensteiner</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://www.uni-hannover.de</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Faculty ITC (Earth Observation Science)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>University of Twente</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Remote Sensing; Photogrammetry; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.utwente.nl</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Geoscience and Remote Sensing</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>TU Delft</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Netherlands</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Remote Sensing; Adjustment &amp; Geodesy</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.tudelft.nl</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Geodesy and Geoinformation (Photogrammetry)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>TU Wien</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Austria</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>LiDAR Mapping; Forest LiDAR</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Norbert Pfeifer</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://www.tuwien.at</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Remote Sensing Laboratories</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>University of Zurich</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Remote Sensing; Forest LiDAR</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://www.uzh.ch</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Finnish Geospatial Research Institute</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>National Land Survey of Finland</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Finland</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Forest LiDAR; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Juha Hyyppä</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://www.maanmittauslaitos.fi</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Digital Photogrammetry Research Group</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Purdue University</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ayman Habib</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://www.purdue.edu</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Geodetic Science</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Ohio State University</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Adjustment &amp; Geodesy; Photogrammetry</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://www.osu.edu</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Geomatics (Civil &amp; Construction Eng.)</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Oregon State University</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>LiDAR Mapping; Photogrammetry</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://oregonstate.edu</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Geomatics Engineering</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>University of Calgary</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Adjustment &amp; Geodesy; LiDAR Mapping; SLAM</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Naser El-Sheimy</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://www.ucalgary.ca</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Geodesy and Geomatics Engineering</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>University of New Brunswick</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Adjustment &amp; Geodesy; Remote Sensing</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://www.unb.ca</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Center for Spatial Information Science</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>University of Tokyo</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Remote Sensing; GeoAI / Deep Learning</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://www.u-tokyo.ac.jp</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>LIESMARS (Surveying, Mapping &amp; RS)</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Wuhan University</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping; Remote Sensing</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Liangpei Zhang; Deren Li</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
         <is>
           <t>https://www.whu.edu.cn</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Aerospace Information Research Institute</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Chinese Academy of Sciences</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Remote Sensing; GeoAI / Deep Learning</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
         <is>
           <t>https://www.cas.cn</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Land Surveying &amp; Geo-Informatics (LSGI)</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Hong Kong Polytechnic University</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Photogrammetry; LiDAR Mapping; Adjustment &amp; Geodesy</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Bo Wu</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>https://www.polyu.edu.hk</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Centre for Remote Imaging, Sensing and Processing</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>National University of Singapore</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Remote Sensing; Image Processing</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
         <is>
           <t>https://www.nus.edu.sg</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Geospatial Engineering (Civil &amp; Env. Eng.)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>UNSW Sydney</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Adjustment &amp; Geodesy; Remote Sensing; Photogrammetry</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
         <is>
           <t>https://www.unsw.edu.au</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Infrastructure Engineering (Geomatics)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>University of Melbourne</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>LiDAR Mapping; Remote Sensing</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
         <is>
           <t>https://www.unimelb.edu.au</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>Check group page</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>Link is the university homepage — replace with the lab page once verified</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Autonomous Vision Group</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>University of Tübingen</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Andreas Geiger</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://uni-tuebingen.de</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Computer Vision Group</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Daniel Cremers</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://www.tum.de</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Computer Vision and Geometry Group</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Computer Vision (2D/3D); SLAM; Photogrammetry</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Marc Pollefeys</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://ethz.ch</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Robotics and Perception Group</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>University of Zurich</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Davide Scaramuzza</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://www.uzh.ch</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Autonomous Systems Lab</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ETH Zurich</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>SLAM; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Roland Siegwart</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://ethz.ch</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="3" t="n"/>
-      <c r="C29" s="3" t="n"/>
-      <c r="D29" s="3" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Dyson Robotics Lab</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Imperial College London</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Andrew Davison</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.imperial.ac.uk</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="2" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Smart Robotics Lab</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Stefan Leutenegger</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.tum.de</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="3" t="n"/>
-      <c r="C31" s="3" t="n"/>
-      <c r="D31" s="3" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Air Lab</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>SLAM; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sebastian Scherer</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Robot Perception Lab</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Carnegie Mellon University</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Michael Kaess</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.cmu.edu</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="3" t="n"/>
-      <c r="C33" s="3" t="n"/>
-      <c r="D33" s="3" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Borglab</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Georgia Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>SLAM; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Frank Dellaert</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.gatech.edu</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Chair of Photogrammetry and Remote Sensing</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Technical University of Munich</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Photogrammetry; Computer Vision (2D/3D)</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Uwe Stilla</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>https://www.tum.de</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>3D Geospatial Data Processing Group (3DGeo)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Heidelberg University</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Bernhard Höfle</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>https://www.uni-heidelberg.de</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="2" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Remote Sensing Image Analysis Group</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Karlsruhe Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Stefan Hinz</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>https://www.kit.edu</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="3" t="n"/>
-      <c r="C37" s="3" t="n"/>
-      <c r="D37" s="3" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Institute of Photogrammetry and Remote Sensing (IPF)</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Karlsruhe Institute of Technology</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Computer Vision (2D/3D); Photogrammetry</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Boris Jutzi; Martin Weinmann</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>https://www.kit.edu</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Institute of Cartography and Geoinformatics</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Leibniz University Hannover</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>GeoAI / Deep Learning; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Monika Sester</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>https://www.uni-hannover.de</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n"/>
-      <c r="B39" s="3" t="n"/>
-      <c r="C39" s="3" t="n"/>
-      <c r="D39" s="3" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>EcoVision Lab</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>University of Zurich</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning; Forest LiDAR</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Jan Dirk Wegner</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>https://www.uzh.ch</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Environmental Computational Science and Earth Observation Lab (ECEO)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>EPFL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Switzerland</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Devis Tuia</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>https://www.epfl.ch</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n"/>
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Image Processing Laboratory (IPL)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>University of Valencia</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Gustau Camps-Valls</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>https://www.uv.es</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Chair of Remote Sensing and Landscape Information Systems</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>University of Freiburg</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Barbara Koch</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>https://www.uni-freiburg.de</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Faculty of Environmental Sciences and Natural Resource Management</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Norwegian University of Life Sciences (NMBU)</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Erik Næsset; Terje Gobakken</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>https://www.nmbu.no</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Department of Forest Sciences</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>University of Helsinki</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Finland</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Forest LiDAR; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Mikko Vastaranta</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>https://www.helsinki.fi</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Department of Biogeochemical Integration</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Max Planck Institute for Biogeochemistry</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Markus Reichstein</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>https://www.bgc-jena.mpg.de</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Center for Geospatial Analytics</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>North Carolina State University</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Environmental Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Ross Meentemeyer</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>https://www.ncsu.edu</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Institute of Geodesy</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>University of Stuttgart</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Germany</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Adjustment &amp; Geodesy</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Nico Sneeuw</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>https://www.uni-stuttgart.de</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Institute of Remote Sensing and Digital Earth (RADI)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Chinese Academy of Sciences</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Huadong Guo</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>https://www.cas.cn</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>School of Geospatial Engineering and Science</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Sun Yat-sen University</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Photogrammetry; Remote Sensing; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>https://www.sysu.edu.cn</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>School of Geographic Sciences</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>East China Normal University</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>https://www.ecnu.edu.cn</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Department of Geoinformatics</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>University of Tokyo</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Remote Sensing; GeoAI / Deep Learning</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ryosuke Shibasaki</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>https://www.u-tokyo.ac.jp</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Department of Infrastructure Engineering</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>University of Melbourne</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://www.unimelb.edu.au</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>School of Civil and Environmental Engineering</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>UNSW Sydney</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Adjustment &amp; Geodesy; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Linlin Ge</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.unsw.edu.au</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Digital Photogrammetry Research Group</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Purdue University</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Jinha Jung</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.purdue.edu</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Geospatial Data Analysis Lab</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>University of Florida</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Photogrammetry; LiDAR Mapping</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Benjamin Wu</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://www.ufl.edu</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Spatial Sciences Institute</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>University of Southern California</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>GeoAI / Deep Learning; Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>https://sci.usc.edu</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Center for LiDAR Information Coordination and Knowledge (CLICK)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>NOAA Coastal Services Center</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>LiDAR Mapping; Environmental Remote Sensing</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>https://coast.noaa.gov</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Check group page</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Seed entry — verify current affiliation and links</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>